<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-02
</commit_message>
<xml_diff>
--- a/HK_Swing_Pattern.xlsx
+++ b/HK_Swing_Pattern.xlsx
@@ -17466,7 +17466,7 @@
         <v>48.296</v>
       </c>
       <c r="AO145" s="2" t="n">
-        <v>51.847</v>
+        <v>51.846</v>
       </c>
       <c r="AP145" s="2" t="n">
         <v>60.085</v>
@@ -18972,7 +18972,7 @@
         <v>0.701</v>
       </c>
       <c r="AN158" s="2" t="n">
-        <v>0.713</v>
+        <v>0.714</v>
       </c>
       <c r="AO158" s="2" t="n">
         <v>0.707</v>
@@ -19088,7 +19088,7 @@
         <v>4.223</v>
       </c>
       <c r="AO159" s="2" t="n">
-        <v>4.23</v>
+        <v>4.229</v>
       </c>
       <c r="AP159" s="2" t="n">
         <v>4.705</v>
@@ -29803,7 +29803,7 @@
         <v>63.274</v>
       </c>
       <c r="AO252" s="2" t="n">
-        <v>63.36</v>
+        <v>63.359</v>
       </c>
       <c r="AP252" s="2" t="n">
         <v>65.73999999999999</v>
@@ -45081,7 +45081,7 @@
         <v>4.751</v>
       </c>
       <c r="AK388" s="2" t="n">
-        <v>4.581</v>
+        <v>4.58</v>
       </c>
       <c r="AL388" s="2" t="n">
         <v>4.702</v>
@@ -54664,7 +54664,7 @@
         <v>33.7</v>
       </c>
       <c r="D472" s="2" t="n">
-        <v>40.4</v>
+        <v>41.22</v>
       </c>
       <c r="E472" s="2" t="inlineStr"/>
       <c r="F472" s="2" t="inlineStr"/>
@@ -57190,7 +57190,7 @@
         <v>8.175000000000001</v>
       </c>
       <c r="AO493" s="2" t="n">
-        <v>7.98</v>
+        <v>7.981</v>
       </c>
       <c r="AP493" s="2" t="n">
         <v>8.795</v>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-04
</commit_message>
<xml_diff>
--- a/HK_Swing_Pattern.xlsx
+++ b/HK_Swing_Pattern.xlsx
@@ -50815,14 +50815,10 @@
       <c r="AC438" s="2" t="n">
         <v>108.2</v>
       </c>
-      <c r="AD438" s="2" t="n">
-        <v>53</v>
-      </c>
+      <c r="AD438" s="2" t="inlineStr"/>
       <c r="AE438" s="2" t="inlineStr"/>
       <c r="AF438" s="2" t="inlineStr"/>
-      <c r="AG438" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AG438" s="2" t="inlineStr"/>
       <c r="AH438" s="2" t="inlineStr"/>
       <c r="AI438" s="2" t="inlineStr">
         <is>

</xml_diff>